<commit_message>
Update from local workspace
</commit_message>
<xml_diff>
--- a/Future Store List.xlsx
+++ b/Future Store List.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8400"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t>Store</t>
   </si>
@@ -216,9 +216,6 @@
   </si>
   <si>
     <t>THRIPUNITHURA FUTURE</t>
-  </si>
-  <si>
-    <t>CHERTHALA FUTURE</t>
   </si>
 </sst>
 </file>
@@ -1401,7 +1398,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A64"/>
+  <dimension ref="A1:A63"/>
   <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="30.712962962963" style="1" customWidth="1"/>
@@ -1718,13 +1715,8 @@
       </c>
     </row>
     <row r="63" spans="1:1">
-      <c r="A63" s="6" t="s">
+      <c r="A63" s="8" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1">
-      <c r="A64" s="8" t="s">
-        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>